<commit_message>
traitement commentaires ypoiron 70fe0779872f8bd3c6b26f7860e51eb6b2f223ed
</commit_message>
<xml_diff>
--- a/cp-ins-iti-105/ig/StructureDefinition-pdsm-simplified-publish.xlsx
+++ b/cp-ins-iti-105/ig/StructureDefinition-pdsm-simplified-publish.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="524">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T12:04:23+00:00</t>
+    <t>2026-10-15T15:21:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -283,7 +283,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}constr-sp-subject-sourcePatientInfo-ins:Lorsque subject.identifier porte un matricule INS et que context.sourcePatientInfo est fourni, la ressource Patient contenue référencée par context.sourcePatientInfo doit porter le même matricule INS (même system et même value). {(subject.identifier.where(system in ('urn:oid:1.2.250.1.213.1.4.8' | 'urn:oid:1.2.250.1.213.1.4.9' | 'urn:oid:1.2.250.1.213.1.4.10' | 'urn:oid:1.2.250.1.213.1.4.11')).exists() and context.sourcePatientInfo.exists()) implies contained.ofType(Patient).where(('#' + id) = %resource.context.sourcePatientInfo.reference).identifier.where(system = %resource.subject.identifier.system and value = %resource.subject.identifier.value).exists()}</t>
   </si>
   <si>
     <t>Event</t>
@@ -861,7 +861,7 @@
 </t>
   </si>
   <si>
-    <t>Patient concerné par ce document. La ressource référencée peut être présente sous l’élément DocumentReference.contained ou via le champ identifier.</t>
+    <t>Patient titulaire du dossier dans le système cible. Lorsque le patient dispose d'une identité INS qualifiée, le matricule INS est porté par subject.identifier (référence logique, admise par IHE MHD ITI-105 §2:3.105.4.1.2.2 pour un identifiant national). La référence peut aussi pointer une ressource Patient déjà connue du système cible. Conformément à IHE MHD, la ressource Patient n'est pas contenue (contained) : les traits du patient tels que connus du producteur sont portés par context.sourcePatientInfo. Lorsque context.sourcePatientInfo est fourni, son matricule INS doit être identique à celui de subject.identifier (invariant constr-sp-subject-sourcePatientInfo-ins) ; en cas de discordance, la transaction est rejetée.</t>
   </si>
   <si>
     <t>Who or what the document is about. The document can be about a person, (patient or healthcare practitioner), a device (e.g. a machine) or even a group of subjects (such as a document about a herd of farm animals, or a set of patients that share a common exposure).</t>
@@ -1635,10 +1635,6 @@
   </si>
   <si>
     <t>The Patient Information as known when the document was published. May be a reference to a version specific, or contained.</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-constr-sp-sourcePatientInfo-contained:Lorsqu'il est fourni, context.sourcePatientInfo doit référencer une ressource Patient contenue (contained), cf spécifications IHE MHD ITI-105 §2:3.105.4.1.2.2. {reference.exists() implies reference.startsWith('#')}</t>
   </si>
   <si>
     <t>DocumentEntry.sourcePatientInfo, DocumentEntry.sourcePatientId</t>
@@ -9744,7 +9740,7 @@
         <v>80</v>
       </c>
       <c r="AJ63" t="s" s="2">
-        <v>514</v>
+        <v>105</v>
       </c>
       <c r="AK63" t="s" s="2">
         <v>80</v>
@@ -9765,15 +9761,15 @@
         <v>80</v>
       </c>
       <c r="AQ63" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9796,16 +9792,16 @@
         <v>80</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>517</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>518</v>
       </c>
-      <c r="M64" t="s" s="2">
+      <c r="N64" t="s" s="2">
         <v>519</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>520</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
@@ -9855,7 +9851,7 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>81</v>
@@ -9873,22 +9869,22 @@
         <v>80</v>
       </c>
       <c r="AL64" t="s" s="2">
+        <v>520</v>
+      </c>
+      <c r="AM64" t="s" s="2">
         <v>521</v>
       </c>
-      <c r="AM64" t="s" s="2">
+      <c r="AN64" t="s" s="2">
         <v>522</v>
       </c>
-      <c r="AN64" t="s" s="2">
+      <c r="AO64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ64" t="s" s="2">
         <v>523</v>
-      </c>
-      <c r="AO64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
-        <v>524</v>
       </c>
     </row>
   </sheetData>

</xml_diff>